<commit_message>
cambiar todas las letras building del derecho al izquierdo
</commit_message>
<xml_diff>
--- a/public/plantilla.xlsx
+++ b/public/plantilla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\cargaHorariav2\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2334DF6-CD04-4E54-A7AF-3CFD27FB3141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501212BF-E2B4-4E43-B57B-D0AEDD042837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,17 +426,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -628,32 +617,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -675,11 +638,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -700,37 +700,88 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -743,19 +794,22 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -790,69 +844,14 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -914,18 +913,18 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>247650</xdr:rowOff>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1828800" cy="847725"/>
+    <xdr:ext cx="1809750" cy="704850"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image4.jpg">
+        <xdr:cNvPr id="4" name="image2.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -951,45 +950,65 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>696686</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>87086</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1809750" cy="704850"/>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2842986</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1128486</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image2.png">
+        <xdr:cNvPr id="5" name="Imagen 4" descr="Gobierno de Michoacán">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{718B394E-4A84-4A64-BE29-D7A6372D2BBB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect t="23392" b="28655"/>
+        <a:stretch/>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
+          <a:off x="16187057" y="87086"/>
+          <a:ext cx="2146300" cy="1041400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1234,13 +1253,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="91.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46"/>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
+      <c r="A1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -1262,15 +1281,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="49"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="31"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
@@ -1292,13 +1311,13 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="52"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="34"/>
       <c r="F3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1324,11 +1343,11 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="44"/>
-      <c r="B4" s="45"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="55"/>
+      <c r="A4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="37"/>
       <c r="F4" s="6" t="s">
         <v>1</v>
       </c>
@@ -1395,7 +1414,7 @@
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
     </row>
-    <row r="6" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>9</v>
       </c>
@@ -1425,7 +1444,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
@@ -1455,7 +1474,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="108.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -1485,7 +1504,7 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="108.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>12</v>
       </c>
@@ -1515,7 +1534,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>13</v>
       </c>
@@ -1545,7 +1564,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>14</v>
       </c>
@@ -1575,7 +1594,7 @@
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>15</v>
       </c>
@@ -1605,7 +1624,7 @@
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" ht="108.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>16</v>
       </c>
@@ -1635,7 +1654,7 @@
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
     </row>
-    <row r="14" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>17</v>
       </c>
@@ -1665,7 +1684,7 @@
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>18</v>
       </c>
@@ -1695,7 +1714,7 @@
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
     </row>
-    <row r="16" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
         <v>19</v>
       </c>
@@ -1725,7 +1744,7 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" ht="109.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>20</v>
       </c>
@@ -1755,7 +1774,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="108.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>21</v>
       </c>
@@ -1786,13 +1805,13 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="50"/>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
+      <c r="A19" s="32"/>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -1814,13 +1833,13 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="121.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="30"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="22"/>
+      <c r="A20" s="50"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="41"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -1842,19 +1861,19 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="39"/>
+      <c r="B21" s="59"/>
       <c r="C21" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="27"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="45"/>
       <c r="F21" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="64"/>
+      <c r="G21" s="15"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
@@ -1876,13 +1895,13 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="40"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="65"/>
+      <c r="A22" s="60"/>
+      <c r="B22" s="61"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -1904,13 +1923,13 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" spans="1:26" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="63"/>
+      <c r="A23" s="52"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="64"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -1932,15 +1951,15 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="16" t="s">
+      <c r="A24" s="54"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="56"/>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="57"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="20"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -1962,13 +1981,13 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="57"/>
+      <c r="A25" s="38"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="20"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
@@ -1990,15 +2009,15 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="56"/>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="57"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="20"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
@@ -2020,13 +2039,13 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="19"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="56"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="57"/>
+      <c r="A27" s="38"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="20"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
@@ -2048,13 +2067,13 @@
       <c r="Z27" s="1"/>
     </row>
     <row r="28" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="28"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="61"/>
+      <c r="A28" s="48"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="23"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
@@ -2078,7 +2097,7 @@
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
-      <c r="C29" s="58"/>
+      <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -8424,7 +8443,12 @@
     <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A21:B22"/>
+    <mergeCell ref="C23:G23"/>
     <mergeCell ref="F21:G22"/>
     <mergeCell ref="C24:G28"/>
     <mergeCell ref="A3:B4"/>
@@ -8434,17 +8458,11 @@
     <mergeCell ref="C3:E4"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F23:G23"/>
     <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C23:E23"/>
     <mergeCell ref="C21:E22"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A21:B22"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.22326454033771001" right="0.22326454033771001" top="0.20731707317073" bottom="0.22326454033771001" header="0" footer="0"/>

</xml_diff>